<commit_message>
ANS-009-015 - Mise à jour du JDV_J264_ModeEtCentreDePriseEnCharge_MDPH (#357)
* 352_354-ContenuCDA_RC-MaJ_JDV_J264

* ErreurScript

* Test

* Update fhir-worklows.yml

* ContenuCDA

* MiseEnForme

---------

Co-authored-by: Eric <146948932+SEBELIN@users.noreply.github.com> 97f6d51de786672379c98ee55dec115d76de808d
</commit_message>
<xml_diff>
--- a/main/ig/StructureDefinition-esms-task.xlsx
+++ b/main/ig/StructureDefinition-esms-task.xlsx
@@ -13,7 +13,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5985" uniqueCount="648">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5985" uniqueCount="647">
   <si>
     <t>Property</t>
   </si>
@@ -54,7 +54,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2026-06-26T14:17:25+00:00</t>
+    <t>2026-06-26T14:37:44+00:00</t>
   </si>
   <si>
     <t>Publisher</t>
@@ -1778,10 +1778,6 @@
   </si>
   <si>
     <t>Permet de définir le mode de prise en charge</t>
-  </si>
-  <si>
-    <t>ele-1:All FHIR elements must have a @value or children {hasValue() or (children().count() &gt; id.count())}
-regle-ModePriseEnCharge:Les codes possibles pour le mode de prise en charge sont : 46 (Hébergement (accueil jour et nuit)) ; 47 (Accueil de jour); 48 (Accueil de nuit) {(value.coding.where(code='48').exists()) or (value.coding.where(code='47').exists()) or (value.coding.where(code='46').exists())}</t>
   </si>
   <si>
     <t>Task.input:modePriseCharge.id</t>
@@ -16111,7 +16107,7 @@
         <v>76</v>
       </c>
       <c r="AJ120" t="s" s="2">
-        <v>554</v>
+        <v>98</v>
       </c>
       <c r="AK120" t="s" s="2">
         <v>76</v>
@@ -16128,7 +16124,7 @@
     </row>
     <row r="121">
       <c r="A121" t="s" s="2">
-        <v>555</v>
+        <v>554</v>
       </c>
       <c r="B121" t="s" s="2">
         <v>440</v>
@@ -16240,7 +16236,7 @@
     </row>
     <row r="122">
       <c r="A122" t="s" s="2">
-        <v>556</v>
+        <v>555</v>
       </c>
       <c r="B122" t="s" s="2">
         <v>441</v>
@@ -16354,7 +16350,7 @@
     </row>
     <row r="123">
       <c r="A123" t="s" s="2">
-        <v>557</v>
+        <v>556</v>
       </c>
       <c r="B123" t="s" s="2">
         <v>442</v>
@@ -16470,7 +16466,7 @@
     </row>
     <row r="124">
       <c r="A124" t="s" s="2">
-        <v>558</v>
+        <v>557</v>
       </c>
       <c r="B124" t="s" s="2">
         <v>443</v>
@@ -16518,7 +16514,7 @@
         <v>76</v>
       </c>
       <c r="S124" t="s" s="2">
-        <v>559</v>
+        <v>558</v>
       </c>
       <c r="T124" t="s" s="2">
         <v>76</v>
@@ -16586,7 +16582,7 @@
     </row>
     <row r="125">
       <c r="A125" t="s" s="2">
-        <v>560</v>
+        <v>559</v>
       </c>
       <c r="B125" t="s" s="2">
         <v>450</v>
@@ -16649,7 +16645,7 @@
       </c>
       <c r="Y125" s="2"/>
       <c r="Z125" t="s" s="2">
-        <v>561</v>
+        <v>560</v>
       </c>
       <c r="AA125" t="s" s="2">
         <v>76</v>
@@ -16696,10 +16692,10 @@
     </row>
     <row r="126">
       <c r="A126" t="s" s="2">
+        <v>561</v>
+      </c>
+      <c r="B126" t="s" s="2">
         <v>562</v>
-      </c>
-      <c r="B126" t="s" s="2">
-        <v>563</v>
       </c>
       <c r="C126" s="2"/>
       <c r="D126" t="s" s="2">
@@ -16808,10 +16804,10 @@
     </row>
     <row r="127">
       <c r="A127" t="s" s="2">
+        <v>563</v>
+      </c>
+      <c r="B127" t="s" s="2">
         <v>564</v>
-      </c>
-      <c r="B127" t="s" s="2">
-        <v>565</v>
       </c>
       <c r="C127" s="2"/>
       <c r="D127" t="s" s="2">
@@ -16922,10 +16918,10 @@
     </row>
     <row r="128">
       <c r="A128" t="s" s="2">
+        <v>565</v>
+      </c>
+      <c r="B128" t="s" s="2">
         <v>566</v>
-      </c>
-      <c r="B128" t="s" s="2">
-        <v>567</v>
       </c>
       <c r="C128" s="2"/>
       <c r="D128" t="s" s="2">
@@ -16951,16 +16947,16 @@
         <v>140</v>
       </c>
       <c r="L128" t="s" s="2">
+        <v>567</v>
+      </c>
+      <c r="M128" t="s" s="2">
         <v>568</v>
       </c>
-      <c r="M128" t="s" s="2">
+      <c r="N128" t="s" s="2">
         <v>569</v>
       </c>
-      <c r="N128" t="s" s="2">
+      <c r="O128" t="s" s="2">
         <v>570</v>
-      </c>
-      <c r="O128" t="s" s="2">
-        <v>571</v>
       </c>
       <c r="P128" t="s" s="2">
         <v>76</v>
@@ -17009,7 +17005,7 @@
         <v>76</v>
       </c>
       <c r="AF128" t="s" s="2">
-        <v>572</v>
+        <v>571</v>
       </c>
       <c r="AG128" t="s" s="2">
         <v>77</v>
@@ -17027,21 +17023,21 @@
         <v>76</v>
       </c>
       <c r="AL128" t="s" s="2">
+        <v>572</v>
+      </c>
+      <c r="AM128" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="AN128" t="s" s="2">
         <v>573</v>
-      </c>
-      <c r="AM128" t="s" s="2">
-        <v>76</v>
-      </c>
-      <c r="AN128" t="s" s="2">
-        <v>574</v>
       </c>
     </row>
     <row r="129">
       <c r="A129" t="s" s="2">
+        <v>574</v>
+      </c>
+      <c r="B129" t="s" s="2">
         <v>575</v>
-      </c>
-      <c r="B129" t="s" s="2">
-        <v>576</v>
       </c>
       <c r="C129" s="2"/>
       <c r="D129" t="s" s="2">
@@ -17067,16 +17063,16 @@
         <v>100</v>
       </c>
       <c r="L129" t="s" s="2">
+        <v>576</v>
+      </c>
+      <c r="M129" t="s" s="2">
         <v>577</v>
       </c>
-      <c r="M129" t="s" s="2">
+      <c r="N129" t="s" s="2">
         <v>578</v>
       </c>
-      <c r="N129" t="s" s="2">
+      <c r="O129" t="s" s="2">
         <v>579</v>
-      </c>
-      <c r="O129" t="s" s="2">
-        <v>580</v>
       </c>
       <c r="P129" t="s" s="2">
         <v>76</v>
@@ -17125,7 +17121,7 @@
         <v>76</v>
       </c>
       <c r="AF129" t="s" s="2">
-        <v>581</v>
+        <v>580</v>
       </c>
       <c r="AG129" t="s" s="2">
         <v>77</v>
@@ -17143,24 +17139,24 @@
         <v>76</v>
       </c>
       <c r="AL129" t="s" s="2">
+        <v>581</v>
+      </c>
+      <c r="AM129" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="AN129" t="s" s="2">
         <v>582</v>
-      </c>
-      <c r="AM129" t="s" s="2">
-        <v>76</v>
-      </c>
-      <c r="AN129" t="s" s="2">
-        <v>583</v>
       </c>
     </row>
     <row r="130">
       <c r="A130" t="s" s="2">
-        <v>584</v>
+        <v>583</v>
       </c>
       <c r="B130" t="s" s="2">
         <v>432</v>
       </c>
       <c r="C130" t="s" s="2">
-        <v>585</v>
+        <v>584</v>
       </c>
       <c r="D130" t="s" s="2">
         <v>433</v>
@@ -17185,7 +17181,7 @@
         <v>403</v>
       </c>
       <c r="L130" t="s" s="2">
-        <v>586</v>
+        <v>585</v>
       </c>
       <c r="M130" t="s" s="2">
         <v>436</v>
@@ -17270,7 +17266,7 @@
     </row>
     <row r="131">
       <c r="A131" t="s" s="2">
-        <v>587</v>
+        <v>586</v>
       </c>
       <c r="B131" t="s" s="2">
         <v>440</v>
@@ -17382,7 +17378,7 @@
     </row>
     <row r="132">
       <c r="A132" t="s" s="2">
-        <v>588</v>
+        <v>587</v>
       </c>
       <c r="B132" t="s" s="2">
         <v>441</v>
@@ -17496,7 +17492,7 @@
     </row>
     <row r="133">
       <c r="A133" t="s" s="2">
-        <v>589</v>
+        <v>588</v>
       </c>
       <c r="B133" t="s" s="2">
         <v>442</v>
@@ -17612,7 +17608,7 @@
     </row>
     <row r="134">
       <c r="A134" t="s" s="2">
-        <v>590</v>
+        <v>589</v>
       </c>
       <c r="B134" t="s" s="2">
         <v>443</v>
@@ -17660,7 +17656,7 @@
         <v>76</v>
       </c>
       <c r="S134" t="s" s="2">
-        <v>591</v>
+        <v>590</v>
       </c>
       <c r="T134" t="s" s="2">
         <v>76</v>
@@ -17728,7 +17724,7 @@
     </row>
     <row r="135">
       <c r="A135" t="s" s="2">
-        <v>592</v>
+        <v>591</v>
       </c>
       <c r="B135" t="s" s="2">
         <v>450</v>
@@ -17791,7 +17787,7 @@
       </c>
       <c r="Y135" s="2"/>
       <c r="Z135" t="s" s="2">
-        <v>593</v>
+        <v>592</v>
       </c>
       <c r="AA135" t="s" s="2">
         <v>76</v>
@@ -17838,13 +17834,13 @@
     </row>
     <row r="136">
       <c r="A136" t="s" s="2">
-        <v>594</v>
+        <v>593</v>
       </c>
       <c r="B136" t="s" s="2">
         <v>432</v>
       </c>
       <c r="C136" t="s" s="2">
-        <v>595</v>
+        <v>594</v>
       </c>
       <c r="D136" t="s" s="2">
         <v>433</v>
@@ -17869,7 +17865,7 @@
         <v>403</v>
       </c>
       <c r="L136" t="s" s="2">
-        <v>596</v>
+        <v>595</v>
       </c>
       <c r="M136" t="s" s="2">
         <v>436</v>
@@ -17954,7 +17950,7 @@
     </row>
     <row r="137">
       <c r="A137" t="s" s="2">
-        <v>597</v>
+        <v>596</v>
       </c>
       <c r="B137" t="s" s="2">
         <v>440</v>
@@ -18066,7 +18062,7 @@
     </row>
     <row r="138">
       <c r="A138" t="s" s="2">
-        <v>598</v>
+        <v>597</v>
       </c>
       <c r="B138" t="s" s="2">
         <v>441</v>
@@ -18180,7 +18176,7 @@
     </row>
     <row r="139">
       <c r="A139" t="s" s="2">
-        <v>599</v>
+        <v>598</v>
       </c>
       <c r="B139" t="s" s="2">
         <v>442</v>
@@ -18296,7 +18292,7 @@
     </row>
     <row r="140">
       <c r="A140" t="s" s="2">
-        <v>600</v>
+        <v>599</v>
       </c>
       <c r="B140" t="s" s="2">
         <v>443</v>
@@ -18344,7 +18340,7 @@
         <v>76</v>
       </c>
       <c r="S140" t="s" s="2">
-        <v>601</v>
+        <v>600</v>
       </c>
       <c r="T140" t="s" s="2">
         <v>76</v>
@@ -18412,7 +18408,7 @@
     </row>
     <row r="141">
       <c r="A141" t="s" s="2">
-        <v>602</v>
+        <v>601</v>
       </c>
       <c r="B141" t="s" s="2">
         <v>450</v>
@@ -18524,13 +18520,13 @@
     </row>
     <row r="142">
       <c r="A142" t="s" s="2">
-        <v>603</v>
+        <v>602</v>
       </c>
       <c r="B142" t="s" s="2">
         <v>432</v>
       </c>
       <c r="C142" t="s" s="2">
-        <v>604</v>
+        <v>603</v>
       </c>
       <c r="D142" t="s" s="2">
         <v>433</v>
@@ -18555,7 +18551,7 @@
         <v>403</v>
       </c>
       <c r="L142" t="s" s="2">
-        <v>605</v>
+        <v>604</v>
       </c>
       <c r="M142" t="s" s="2">
         <v>436</v>
@@ -18640,7 +18636,7 @@
     </row>
     <row r="143">
       <c r="A143" t="s" s="2">
-        <v>606</v>
+        <v>605</v>
       </c>
       <c r="B143" t="s" s="2">
         <v>440</v>
@@ -18752,7 +18748,7 @@
     </row>
     <row r="144">
       <c r="A144" t="s" s="2">
-        <v>607</v>
+        <v>606</v>
       </c>
       <c r="B144" t="s" s="2">
         <v>441</v>
@@ -18866,7 +18862,7 @@
     </row>
     <row r="145">
       <c r="A145" t="s" s="2">
-        <v>608</v>
+        <v>607</v>
       </c>
       <c r="B145" t="s" s="2">
         <v>442</v>
@@ -18982,7 +18978,7 @@
     </row>
     <row r="146">
       <c r="A146" t="s" s="2">
-        <v>609</v>
+        <v>608</v>
       </c>
       <c r="B146" t="s" s="2">
         <v>443</v>
@@ -19030,7 +19026,7 @@
         <v>76</v>
       </c>
       <c r="S146" t="s" s="2">
-        <v>610</v>
+        <v>609</v>
       </c>
       <c r="T146" t="s" s="2">
         <v>76</v>
@@ -19098,7 +19094,7 @@
     </row>
     <row r="147">
       <c r="A147" t="s" s="2">
-        <v>611</v>
+        <v>610</v>
       </c>
       <c r="B147" t="s" s="2">
         <v>450</v>
@@ -19127,7 +19123,7 @@
         <v>243</v>
       </c>
       <c r="L147" t="s" s="2">
-        <v>612</v>
+        <v>611</v>
       </c>
       <c r="M147" t="s" s="2">
         <v>453</v>
@@ -19161,7 +19157,7 @@
       </c>
       <c r="Y147" s="2"/>
       <c r="Z147" t="s" s="2">
-        <v>613</v>
+        <v>612</v>
       </c>
       <c r="AA147" t="s" s="2">
         <v>76</v>
@@ -19208,13 +19204,13 @@
     </row>
     <row r="148">
       <c r="A148" t="s" s="2">
-        <v>614</v>
+        <v>613</v>
       </c>
       <c r="B148" t="s" s="2">
         <v>432</v>
       </c>
       <c r="C148" t="s" s="2">
-        <v>615</v>
+        <v>614</v>
       </c>
       <c r="D148" t="s" s="2">
         <v>433</v>
@@ -19239,7 +19235,7 @@
         <v>403</v>
       </c>
       <c r="L148" t="s" s="2">
-        <v>616</v>
+        <v>615</v>
       </c>
       <c r="M148" t="s" s="2">
         <v>436</v>
@@ -19324,7 +19320,7 @@
     </row>
     <row r="149">
       <c r="A149" t="s" s="2">
-        <v>617</v>
+        <v>616</v>
       </c>
       <c r="B149" t="s" s="2">
         <v>440</v>
@@ -19436,7 +19432,7 @@
     </row>
     <row r="150">
       <c r="A150" t="s" s="2">
-        <v>618</v>
+        <v>617</v>
       </c>
       <c r="B150" t="s" s="2">
         <v>441</v>
@@ -19550,7 +19546,7 @@
     </row>
     <row r="151">
       <c r="A151" t="s" s="2">
-        <v>619</v>
+        <v>618</v>
       </c>
       <c r="B151" t="s" s="2">
         <v>442</v>
@@ -19666,7 +19662,7 @@
     </row>
     <row r="152">
       <c r="A152" t="s" s="2">
-        <v>620</v>
+        <v>619</v>
       </c>
       <c r="B152" t="s" s="2">
         <v>443</v>
@@ -19714,7 +19710,7 @@
         <v>76</v>
       </c>
       <c r="S152" t="s" s="2">
-        <v>621</v>
+        <v>620</v>
       </c>
       <c r="T152" t="s" s="2">
         <v>76</v>
@@ -19782,7 +19778,7 @@
     </row>
     <row r="153">
       <c r="A153" t="s" s="2">
-        <v>622</v>
+        <v>621</v>
       </c>
       <c r="B153" t="s" s="2">
         <v>450</v>
@@ -19894,13 +19890,13 @@
     </row>
     <row r="154">
       <c r="A154" t="s" s="2">
-        <v>623</v>
+        <v>622</v>
       </c>
       <c r="B154" t="s" s="2">
         <v>432</v>
       </c>
       <c r="C154" t="s" s="2">
-        <v>624</v>
+        <v>623</v>
       </c>
       <c r="D154" t="s" s="2">
         <v>433</v>
@@ -19925,7 +19921,7 @@
         <v>403</v>
       </c>
       <c r="L154" t="s" s="2">
-        <v>625</v>
+        <v>624</v>
       </c>
       <c r="M154" t="s" s="2">
         <v>436</v>
@@ -20010,7 +20006,7 @@
     </row>
     <row r="155">
       <c r="A155" t="s" s="2">
-        <v>626</v>
+        <v>625</v>
       </c>
       <c r="B155" t="s" s="2">
         <v>440</v>
@@ -20122,7 +20118,7 @@
     </row>
     <row r="156">
       <c r="A156" t="s" s="2">
-        <v>627</v>
+        <v>626</v>
       </c>
       <c r="B156" t="s" s="2">
         <v>441</v>
@@ -20236,7 +20232,7 @@
     </row>
     <row r="157">
       <c r="A157" t="s" s="2">
-        <v>628</v>
+        <v>627</v>
       </c>
       <c r="B157" t="s" s="2">
         <v>442</v>
@@ -20352,7 +20348,7 @@
     </row>
     <row r="158">
       <c r="A158" t="s" s="2">
-        <v>629</v>
+        <v>628</v>
       </c>
       <c r="B158" t="s" s="2">
         <v>443</v>
@@ -20400,7 +20396,7 @@
         <v>76</v>
       </c>
       <c r="S158" t="s" s="2">
-        <v>630</v>
+        <v>629</v>
       </c>
       <c r="T158" t="s" s="2">
         <v>76</v>
@@ -20468,7 +20464,7 @@
     </row>
     <row r="159">
       <c r="A159" t="s" s="2">
-        <v>631</v>
+        <v>630</v>
       </c>
       <c r="B159" t="s" s="2">
         <v>450</v>
@@ -20580,10 +20576,10 @@
     </row>
     <row r="160">
       <c r="A160" t="s" s="2">
-        <v>632</v>
+        <v>631</v>
       </c>
       <c r="B160" t="s" s="2">
-        <v>632</v>
+        <v>631</v>
       </c>
       <c r="C160" s="2"/>
       <c r="D160" t="s" s="2">
@@ -20609,14 +20605,14 @@
         <v>403</v>
       </c>
       <c r="L160" t="s" s="2">
+        <v>632</v>
+      </c>
+      <c r="M160" t="s" s="2">
         <v>633</v>
-      </c>
-      <c r="M160" t="s" s="2">
-        <v>634</v>
       </c>
       <c r="N160" s="2"/>
       <c r="O160" t="s" s="2">
-        <v>635</v>
+        <v>634</v>
       </c>
       <c r="P160" t="s" s="2">
         <v>76</v>
@@ -20665,7 +20661,7 @@
         <v>76</v>
       </c>
       <c r="AF160" t="s" s="2">
-        <v>632</v>
+        <v>631</v>
       </c>
       <c r="AG160" t="s" s="2">
         <v>77</v>
@@ -20694,10 +20690,10 @@
     </row>
     <row r="161">
       <c r="A161" t="s" s="2">
-        <v>636</v>
+        <v>635</v>
       </c>
       <c r="B161" t="s" s="2">
-        <v>636</v>
+        <v>635</v>
       </c>
       <c r="C161" s="2"/>
       <c r="D161" t="s" s="2">
@@ -20806,10 +20802,10 @@
     </row>
     <row r="162">
       <c r="A162" t="s" s="2">
-        <v>637</v>
+        <v>636</v>
       </c>
       <c r="B162" t="s" s="2">
-        <v>637</v>
+        <v>636</v>
       </c>
       <c r="C162" s="2"/>
       <c r="D162" t="s" s="2">
@@ -20920,10 +20916,10 @@
     </row>
     <row r="163">
       <c r="A163" t="s" s="2">
-        <v>638</v>
+        <v>637</v>
       </c>
       <c r="B163" t="s" s="2">
-        <v>638</v>
+        <v>637</v>
       </c>
       <c r="C163" s="2"/>
       <c r="D163" t="s" s="2">
@@ -21036,10 +21032,10 @@
     </row>
     <row r="164">
       <c r="A164" t="s" s="2">
-        <v>639</v>
+        <v>638</v>
       </c>
       <c r="B164" t="s" s="2">
-        <v>639</v>
+        <v>638</v>
       </c>
       <c r="C164" s="2"/>
       <c r="D164" t="s" s="2">
@@ -21065,14 +21061,14 @@
         <v>243</v>
       </c>
       <c r="L164" t="s" s="2">
+        <v>639</v>
+      </c>
+      <c r="M164" t="s" s="2">
         <v>640</v>
-      </c>
-      <c r="M164" t="s" s="2">
-        <v>641</v>
       </c>
       <c r="N164" s="2"/>
       <c r="O164" t="s" s="2">
-        <v>642</v>
+        <v>641</v>
       </c>
       <c r="P164" t="s" s="2">
         <v>76</v>
@@ -21100,7 +21096,7 @@
         <v>152</v>
       </c>
       <c r="Y164" t="s" s="2">
-        <v>643</v>
+        <v>642</v>
       </c>
       <c r="Z164" t="s" s="2">
         <v>76</v>
@@ -21121,7 +21117,7 @@
         <v>76</v>
       </c>
       <c r="AF164" t="s" s="2">
-        <v>639</v>
+        <v>638</v>
       </c>
       <c r="AG164" t="s" s="2">
         <v>86</v>
@@ -21150,10 +21146,10 @@
     </row>
     <row r="165">
       <c r="A165" t="s" s="2">
-        <v>644</v>
+        <v>643</v>
       </c>
       <c r="B165" t="s" s="2">
-        <v>644</v>
+        <v>643</v>
       </c>
       <c r="C165" s="2"/>
       <c r="D165" t="s" s="2">
@@ -21179,14 +21175,14 @@
         <v>451</v>
       </c>
       <c r="L165" t="s" s="2">
+        <v>644</v>
+      </c>
+      <c r="M165" t="s" s="2">
         <v>645</v>
-      </c>
-      <c r="M165" t="s" s="2">
-        <v>646</v>
       </c>
       <c r="N165" s="2"/>
       <c r="O165" t="s" s="2">
-        <v>647</v>
+        <v>646</v>
       </c>
       <c r="P165" t="s" s="2">
         <v>76</v>
@@ -21235,7 +21231,7 @@
         <v>76</v>
       </c>
       <c r="AF165" t="s" s="2">
-        <v>644</v>
+        <v>643</v>
       </c>
       <c r="AG165" t="s" s="2">
         <v>86</v>

</xml_diff>